<commit_message>
docs: added the report pdf
</commit_message>
<xml_diff>
--- a/docs/statistics.xlsx
+++ b/docs/statistics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Feup\3ANO\RCOM\lab1-code-25-26-deniz\lab1-code-25-26\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9D6B182-C9BA-4516-9045-EF862085F23F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE8DCA81-DE08-4A68-9067-A4C5C0E5B863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EADB7CA2-938E-4F7B-80E6-BB7B094AF1A6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EADB7CA2-938E-4F7B-80E6-BB7B094AF1A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -144,7 +144,37 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
@@ -154,7 +184,7 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Measured, Baud = 9600</c:v>
+            <c:v>Baud x Efficiency</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
@@ -170,36 +200,36 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$F$2:$F$4</c:f>
+              <c:f>(Sheet1!$B$2,Sheet1!$B$5,Sheet1!$B$8)</c:f>
               <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>9600</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.14500000000000002</c:v>
+                  <c:v>38400</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.32500000000000001</c:v>
+                  <c:v>115200</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$I$2:$I$4</c:f>
+              <c:f>(Sheet1!$I$2,Sheet1!$I$5,Sheet1!$I$8)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.77530282191565614</c:v>
+                  <c:v>0.77908545936719842</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.55665845118373358</c:v>
+                  <c:v>0.7786023049354186</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.36965744887665791</c:v>
+                  <c:v>0.76513809821828305</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -207,317 +237,11 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9C1C-4C1F-A168-B11DB25534EF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>Measured, Baud = 38400</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$5:$F$7</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.14500000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.32500000000000001</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$I$5:$I$7</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0.7863945821715228</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.35947257428772122</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>8.962301578663337E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-9C1C-4C1F-A168-B11DB25534EF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>Measured, Baud = 115200</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$8:$F$10</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.14500000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.32500000000000001</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$I$8:$I$10</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0.76534875954885617</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.11956127656699965</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.6241046764427827E-2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-9C1C-4C1F-A168-B11DB25534EF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:v>Theoretical, Baud = 9600</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$2:$F$4</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.14500000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.32500000000000001</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$K$2:$K$4</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.80660377358490565</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.58695652173913049</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-9C1C-4C1F-A168-B11DB25534EF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="4"/>
-          <c:tx>
-            <c:v>Theoretical, Baud = 38400</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent5"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$5:$F$7</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.14500000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.32500000000000001</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$K$5:$K$7</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.68951612903225801</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.421875</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-9C1C-4C1F-A168-B11DB25534EF}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="5"/>
-          <c:order val="5"/>
-          <c:tx>
-            <c:v>Theoretical, Baud = 115200</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$8:$F$10</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.14500000000000002</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.32500000000000001</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$K$8:$K$10</c:f>
-              <c:numCache>
-                <c:formatCode>0.00E+00</c:formatCode>
-                <c:ptCount val="3"/>
-                <c:pt idx="0">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.49709302325581395</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.2410714285714286</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="1"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-9C1C-4C1F-A168-B11DB25534EF}"/>
+              <c16:uniqueId val="{00000000-97ED-48B0-B471-76CC88BDF5F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -525,11 +249,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1522189936"/>
-        <c:axId val="1522206736"/>
+        <c:axId val="743705167"/>
+        <c:axId val="743701327"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1522189936"/>
+        <c:axId val="743705167"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -549,66 +273,310 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>FER (Frame</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" baseline="0"/>
-                  <a:t> Error Ratio)</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="743701327"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="743701327"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
           <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="743705167"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>FER x Efficiency</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>(Sheet1!$F$2,Sheet1!$F$3,Sheet1!$F$6,Sheet1!$F$9)</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.14500000000000002</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.32500000000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.55000000000000004</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>(Sheet1!$I$2,Sheet1!$I$3,Sheet1!$I$6,Sheet1!$I$9)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.77908545936719842</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.71449381982388904</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.37722585956731453</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.36105431177261033</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-4B7C-4C09-BC83-6660DD837330}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="743702767"/>
+        <c:axId val="743719567"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="743702767"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
         <c:numFmt formatCode="0.00E+00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -646,12 +614,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1522206736"/>
+        <c:crossAx val="743719567"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1522206736"/>
+        <c:axId val="743719567"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -671,61 +639,6 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Efficiency</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -763,7 +676,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1522189936"/>
+        <c:crossAx val="743702767"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -775,8 +688,65 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -790,7 +760,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -805,7 +775,223 @@
           <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
-    </c:legend>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Prop Ratio (a) x Efficiency</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>(Sheet1!$G$2,Sheet1!$G$4,Sheet1!$G$7,Sheet1!$G$10)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.03</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.4999999999999997E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>(Sheet1!$I$2,Sheet1!$I$4,Sheet1!$I$7,Sheet1!$I$10)</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.77908545936719842</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.74618786985895735</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.71091575360531123</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.62378991410876972</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8102-47BB-9385-87A1C17B0682}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="257962031"/>
+        <c:axId val="257961071"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="257962031"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="257961071"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="257961071"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="257962031"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -890,6 +1076,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1406,27 +1672,1059 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>22412</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>22412</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>487456</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>90768</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1210235</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>67235</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1176618</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>67236</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30CCA987-CD1A-6526-1C79-F68BFF73BDFE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09EF26C4-6F13-FE26-4810-448968AA9CBF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1439,6 +2737,78 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>168088</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>90767</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>425824</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>67235</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5059279E-88A0-6501-2032-8E1AFD25973A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>79561</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>235324</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>67234</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F361FB7-F268-4445-B229-2148FC588BD7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1846,14 +3216,14 @@
       </c>
       <c r="H2">
         <f>$A$13*8/J2</f>
-        <v>7442.9070903902993</v>
+        <v>7479.2204099251048</v>
       </c>
       <c r="I2">
         <f>H2/B2</f>
-        <v>0.77530282191565614</v>
+        <v>0.77908545936719842</v>
       </c>
       <c r="J2">
-        <v>11.788942</v>
+        <v>11.731704000000001</v>
       </c>
       <c r="K2" s="1">
         <f>(1-F2)/(1+ (2*G2))</f>
@@ -1869,7 +3239,7 @@
         <v>9600</v>
       </c>
       <c r="C3">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="D3" s="1">
         <v>0.05</v>
@@ -1883,22 +3253,22 @@
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G10" si="2">C3/1000 / ((A3*8)/B3)</f>
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H10" si="3">$A$13*8/J3</f>
-        <v>5343.9211313638425</v>
+        <v>6859.1406703093344</v>
       </c>
       <c r="I3">
         <f t="shared" ref="I3:I10" si="4">H3/B3</f>
-        <v>0.55665845118373358</v>
+        <v>0.71449381982388904</v>
       </c>
       <c r="J3">
-        <v>16.419404</v>
+        <v>12.792273</v>
       </c>
       <c r="K3" s="1">
         <f t="shared" ref="K3:K10" si="5">(1-F3)/(1+ (2*G3))</f>
-        <v>0.80660377358490565</v>
+        <v>0.85499999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1910,36 +3280,36 @@
         <v>9600</v>
       </c>
       <c r="C4">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="D4" s="1">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1">
         <f t="shared" si="0"/>
-        <v>0.32500000000000001</v>
+        <v>0</v>
       </c>
       <c r="G4">
         <f t="shared" si="2"/>
-        <v>7.4999999999999997E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="H4">
         <f t="shared" si="3"/>
-        <v>3548.7115092159161</v>
+        <v>7163.4035506459904</v>
       </c>
       <c r="I4">
         <f t="shared" si="4"/>
-        <v>0.36965744887665791</v>
+        <v>0.74618786985895735</v>
       </c>
       <c r="J4">
-        <v>24.725594000000001</v>
+        <v>12.248926000000001</v>
       </c>
       <c r="K4" s="1">
         <f t="shared" si="5"/>
-        <v>0.58695652173913049</v>
+        <v>0.970873786407767</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1969,14 +3339,14 @@
       </c>
       <c r="H5">
         <f t="shared" si="3"/>
-        <v>30197.551955386476</v>
+        <v>29898.328509520074</v>
       </c>
       <c r="I5">
         <f t="shared" si="4"/>
-        <v>0.7863945821715228</v>
+        <v>0.7786023049354186</v>
       </c>
       <c r="J5">
-        <v>2.9056660000000001</v>
+        <v>2.9347460000000001</v>
       </c>
       <c r="K5" s="1">
         <f t="shared" si="5"/>
@@ -1989,39 +3359,39 @@
         <v>8000</v>
       </c>
       <c r="B6" s="2">
-        <v>38400</v>
+        <v>9600</v>
       </c>
       <c r="C6">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="E6">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="F6" s="1">
         <f t="shared" si="0"/>
-        <v>0.14500000000000002</v>
+        <v>0.32500000000000001</v>
       </c>
       <c r="G6">
         <f t="shared" si="2"/>
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <f t="shared" si="3"/>
-        <v>13803.746852648495</v>
+        <v>3621.3682518462192</v>
       </c>
       <c r="I6">
         <f t="shared" si="4"/>
-        <v>0.35947257428772122</v>
+        <v>0.37722585956731453</v>
       </c>
       <c r="J6">
-        <v>6.356535</v>
+        <v>24.229516</v>
       </c>
       <c r="K6" s="1">
         <f t="shared" si="5"/>
-        <v>0.68951612903225801</v>
+        <v>0.67500000000000004</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -2030,39 +3400,39 @@
         <v>8000</v>
       </c>
       <c r="B7" s="2">
-        <v>38400</v>
+        <v>9600</v>
       </c>
       <c r="C7">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="D7" s="1">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F7" s="1">
         <f t="shared" si="0"/>
-        <v>0.32500000000000001</v>
+        <v>0</v>
       </c>
       <c r="G7">
         <f t="shared" si="2"/>
-        <v>0.3</v>
+        <v>0.03</v>
       </c>
       <c r="H7">
         <f t="shared" si="3"/>
-        <v>3441.5238062067215</v>
+        <v>6824.7912346109879</v>
       </c>
       <c r="I7">
         <f t="shared" si="4"/>
-        <v>8.962301578663337E-2</v>
+        <v>0.71091575360531123</v>
       </c>
       <c r="J7">
-        <v>25.495683</v>
+        <v>12.856657</v>
       </c>
       <c r="K7" s="1">
         <f t="shared" si="5"/>
-        <v>0.421875</v>
+        <v>0.94339622641509424</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -2092,14 +3462,14 @@
       </c>
       <c r="H8">
         <f t="shared" si="3"/>
-        <v>88168.177100028232</v>
+        <v>88143.908914746207</v>
       </c>
       <c r="I8">
         <f t="shared" si="4"/>
-        <v>0.76534875954885617</v>
+        <v>0.76513809821828305</v>
       </c>
       <c r="J8">
-        <v>0.99518899999999999</v>
+        <v>0.99546299999999999</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" si="5"/>
@@ -2112,39 +3482,39 @@
         <v>8000</v>
       </c>
       <c r="B9">
-        <v>115200</v>
+        <v>9600</v>
       </c>
       <c r="C9">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="D9" s="1">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="E9">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="F9" s="1">
         <f t="shared" si="0"/>
-        <v>0.14500000000000002</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="G9">
         <f t="shared" si="2"/>
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="H9">
         <f t="shared" si="3"/>
-        <v>13773.45906051836</v>
+        <v>3466.1213930170593</v>
       </c>
       <c r="I9">
         <f t="shared" si="4"/>
-        <v>0.11956127656699965</v>
+        <v>0.36105431177261033</v>
       </c>
       <c r="J9">
-        <v>6.3705129999999999</v>
+        <v>25.314751000000001</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" si="5"/>
-        <v>0.49709302325581395</v>
+        <v>0.44999999999999996</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -2153,39 +3523,39 @@
         <v>8000</v>
       </c>
       <c r="B10">
-        <v>115200</v>
+        <v>9600</v>
       </c>
       <c r="C10">
         <v>500</v>
       </c>
       <c r="D10" s="1">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1">
         <f>D10+E10*(1-D10)</f>
-        <v>0.32500000000000001</v>
+        <v>0</v>
       </c>
       <c r="G10">
         <f t="shared" si="2"/>
-        <v>0.89999999999999991</v>
+        <v>7.4999999999999997E-2</v>
       </c>
       <c r="H10">
         <f t="shared" si="3"/>
-        <v>3022.9685872620857</v>
+        <v>5988.383175444189</v>
       </c>
       <c r="I10">
         <f t="shared" si="4"/>
-        <v>2.6241046764427827E-2</v>
+        <v>0.62378991410876972</v>
       </c>
       <c r="J10">
-        <v>29.025773000000001</v>
+        <v>14.652369</v>
       </c>
       <c r="K10" s="1">
         <f t="shared" si="5"/>
-        <v>0.2410714285714286</v>
+        <v>0.86956521739130443</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>